<commit_message>
MS Project tracking-instruks også som PDF + oppdatert saksnummer
</commit_message>
<xml_diff>
--- a/03 - Gjennomføring/MS Project tracking-instruks.xlsx
+++ b/03 - Gjennomføring/MS Project tracking-instruks.xlsx
@@ -606,7 +606,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>DEL B — APPLISER CRASHING (NHB-IRGESUND-vedtak)</t>
+          <t>DEL B — APPLISER CRASHING (NHB-2026-15-vedtak)</t>
         </is>
       </c>
     </row>
@@ -2107,7 +2107,7 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>Crashing-endring på 4.1 Råbygg (NHB-IRGESUND)</t>
+          <t>Crashing-endring på 4.1 Råbygg (NHB-2026-15)</t>
         </is>
       </c>
     </row>
@@ -2285,7 +2285,7 @@
       </c>
       <c r="C12" s="21" t="inlineStr">
         <is>
-          <t>Kommunestyret sak NHB-IRGESUND</t>
+          <t>Kommunestyret sak NHB-2026-15</t>
         </is>
       </c>
       <c r="D12" s="21" t="inlineStr">
@@ -2307,7 +2307,7 @@
       </c>
       <c r="C13" s="21" t="inlineStr">
         <is>
-          <t>Endringsdokument NHB-IRGESUND - Schedule crashing.docx</t>
+          <t>Endringsdokument NHB-2026-15 - Schedule crashing.docx</t>
         </is>
       </c>
       <c r="D13" s="21" t="inlineStr">

</xml_diff>